<commit_message>
Update Excel file references to use inputDataGiant.xlsx and remove commented-out optimal routing code
</commit_message>
<xml_diff>
--- a/inputData/inputDataBig.xlsx
+++ b/inputData/inputDataBig.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sillewiberg/Desktop/Skole/Speciale/Master-Thesis-eVTOL-1/inputData/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kapta\Documents\DTU\Speciale\GitHubFiles\inputData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{807D108D-5F36-D74B-B4D3-A6C8B4B741D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37525185-01B2-4036-9C3B-3B2C2188F01B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16340" xr2:uid="{63F903F0-DEEC-1344-9131-28787FF511C5}"/>
+    <workbookView xWindow="7740" yWindow="0" windowWidth="11460" windowHeight="11280" xr2:uid="{63F903F0-DEEC-1344-9131-28787FF511C5}"/>
   </bookViews>
   <sheets>
     <sheet name="PlaneData" sheetId="7" r:id="rId1"/>
@@ -100,13 +100,13 @@
     <t>stopover_allowed</t>
   </si>
   <si>
-    <t>coordinates_kbh</t>
-  </si>
-  <si>
     <t>Plane ID</t>
   </si>
   <si>
     <t>Base Vertiport</t>
+  </si>
+  <si>
+    <t>coordinates</t>
   </si>
 </sst>
 </file>
@@ -514,17 +514,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A94FE46B-0EE8-4D7E-956E-06AD6DDE4FF5}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16"/>
+  <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="16"/>
   <cols>
     <col min="2" max="2" width="12.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" t="s">
         <v>21</v>
-      </c>
-      <c r="B1" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="2" spans="1:2">
@@ -567,7 +567,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3245F359-CA05-2247-86C6-92433A84B0A2}">
   <dimension ref="A1:F20"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="16"/>
   <cols>
     <col min="3" max="3" width="22.5" customWidth="1"/>
     <col min="4" max="4" width="13.33203125" bestFit="1" customWidth="1"/>
@@ -585,7 +585,7 @@
         <v>3</v>
       </c>
       <c r="D1" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="2" spans="1:6">
@@ -688,7 +688,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0891C305-141D-384C-BB9E-30507F3FCDCC}">
   <dimension ref="A1:X32"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="16"/>
   <cols>
     <col min="5" max="5" width="11.83203125" customWidth="1"/>
     <col min="6" max="6" width="11.5" customWidth="1"/>

</xml_diff>